<commit_message>
Fix WIP/JMC bulk import bugs: correctly handle typo 'discription' and prevent false header matching on 'sr.' locations
</commit_message>
<xml_diff>
--- a/frontend/public/jmc_bulk_upload_sample.xlsx
+++ b/frontend/public/jmc_bulk_upload_sample.xlsx
@@ -398,10 +398,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F24"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="B1" t="str">
-        <v xml:space="preserve">Name Of Circle : </v>
+        <v>Name Of Circle :</v>
       </c>
       <c r="D1" t="str">
         <v>SOLAN</v>
@@ -414,13 +422,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Name Of Circle :</v>
+      <c r="B2" t="str">
+        <v>Name Of Sub Circle :</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="str">
-        <v xml:space="preserve">Name Of Division : </v>
+        <v>Name Of Division :</v>
       </c>
       <c r="D3" t="str">
         <v>SOLAN</v>
@@ -434,7 +451,7 @@
     </row>
     <row r="4">
       <c r="B4" t="str">
-        <v xml:space="preserve">Name Of Sub/Division :  </v>
+        <v>Name Of Sub/Division :</v>
       </c>
       <c r="D4" t="str">
         <v>ARKI</v>
@@ -448,7 +465,7 @@
     </row>
     <row r="5">
       <c r="B5" t="str">
-        <v xml:space="preserve">Name Of Sub/Station :  </v>
+        <v>Name Of Sub/Station :</v>
       </c>
       <c r="D5" t="str">
         <v>33/11 KV ARKI</v>
@@ -462,7 +479,7 @@
     </row>
     <row r="6">
       <c r="B6" t="str">
-        <v xml:space="preserve">Name Of Feeder :  </v>
+        <v>Name Of Feeder :</v>
       </c>
       <c r="D6" t="str">
         <v>11 KV FEEDER NO.1</v>
@@ -476,7 +493,7 @@
     </row>
     <row r="7">
       <c r="B7" t="str">
-        <v xml:space="preserve">Location : </v>
+        <v>Location :</v>
       </c>
       <c r="D7" t="str">
         <v>ARKI TOWN</v>
@@ -490,7 +507,7 @@
     </row>
     <row r="8">
       <c r="B8" t="str">
-        <v xml:space="preserve">Drawing No :  </v>
+        <v>Drawing No :</v>
       </c>
       <c r="D8" t="str">
         <v>101A</v>

</xml_diff>